<commit_message>
feat(core): cut the demo profiles to five and add a team summary
Two Sales Admins (Nurul Aina, Farah Izzati) replace seven. The generator
still makes one draw per booking for the sales owner, so every other
seeded value is unchanged: Nurul Aina owns 77 bookings, Farah Izzati 71.
The Manager is Robert Khoo. teamSummary counts, per staff profile, the
open bookings whose next move sits with them, by the same rule the
Manager's follow-ups use.

Refs #86

Claude-Session: https://claude.ai/code/session_017h48pattBF2tXyEm7GiAN2
</commit_message>
<xml_diff>
--- a/frontend/public/booking-sheet-template.xlsx
+++ b/frontend/public/booking-sheet-template.xlsx
@@ -86,9 +86,6 @@
     <t>+60 00-000 0102</t>
   </si>
   <si>
-    <t>Kelvin Chow</t>
-  </si>
-  <si>
     <t>Kuan &amp; Teh Advocates</t>
   </si>
   <si>
@@ -104,7 +101,7 @@
     <t>+60 00-000 0103</t>
   </si>
   <si>
-    <t>Dinesh Rao</t>
+    <t>Nurul Aina</t>
   </si>
   <si>
     <t>Devan &amp; Partners</t>
@@ -465,24 +462,24 @@
         <v>1</v>
       </c>
       <c r="J6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="E7" s="6">
         <v>575500</v>
@@ -500,10 +497,10 @@
         <v>0</v>
       </c>
       <c r="J7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -525,7 +522,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -533,7 +530,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -542,27 +539,27 @@
     <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>35</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>37</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>38</v>
       </c>
       <c r="D5" s="0" t="s">
         <v>13</v>
@@ -570,13 +567,13 @@
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>39</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>40</v>
       </c>
       <c r="D6" s="0" t="s">
         <v>14</v>
@@ -584,13 +581,13 @@
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>41</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>42</v>
       </c>
       <c r="D7" s="0" t="s">
         <v>15</v>
@@ -598,13 +595,13 @@
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>44</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>16</v>
@@ -612,44 +609,44 @@
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="12" t="s">
+      <c r="D9" s="0" t="s">
         <v>46</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="12" t="s">
+      <c r="D10" s="0" t="s">
         <v>49</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="12" t="s">
+      <c r="D11" s="0" t="s">
         <v>52</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="12">
@@ -657,13 +654,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="D12" s="0" t="s">
         <v>55</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -671,13 +668,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C13" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="0" t="s">
         <v>57</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="14">
@@ -685,10 +682,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D14" s="0" t="s">
         <v>17</v>
@@ -699,10 +696,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D15" s="0" t="s">
         <v>18</v>
@@ -711,7 +708,7 @@
     <row r="16"/>
     <row r="17">
       <c r="A17" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>

</xml_diff>

<commit_message>
feat(app): redesign Today, Team, the profile menu and Forecast (#87)
Every persona gets the same Today, with the work queue first and a rail beside it. The Manager gets Decisions For You and a Team page at /team, the top bar gets a profile menu, the demo profiles drop to five, and Forecast gets the #54 document stack back with motifs and Ask MortarAI. The docs, README, landing screenshots, pitch script and deck follow, and the graph is refreshed.

Closes #86

Claude-Session: https://claude.ai/code/session_017h48pattBF2tXyEm7GiAN2
</commit_message>
<xml_diff>
--- a/frontend/public/booking-sheet-template.xlsx
+++ b/frontend/public/booking-sheet-template.xlsx
@@ -86,9 +86,6 @@
     <t>+60 00-000 0102</t>
   </si>
   <si>
-    <t>Kelvin Chow</t>
-  </si>
-  <si>
     <t>Kuan &amp; Teh Advocates</t>
   </si>
   <si>
@@ -104,7 +101,7 @@
     <t>+60 00-000 0103</t>
   </si>
   <si>
-    <t>Dinesh Rao</t>
+    <t>Nurul Aina</t>
   </si>
   <si>
     <t>Devan &amp; Partners</t>
@@ -465,24 +462,24 @@
         <v>1</v>
       </c>
       <c r="J6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="E7" s="6">
         <v>575500</v>
@@ -500,10 +497,10 @@
         <v>0</v>
       </c>
       <c r="J7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -525,7 +522,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -533,7 +530,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -542,27 +539,27 @@
     <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>35</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>37</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>38</v>
       </c>
       <c r="D5" s="0" t="s">
         <v>13</v>
@@ -570,13 +567,13 @@
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>39</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>40</v>
       </c>
       <c r="D6" s="0" t="s">
         <v>14</v>
@@ -584,13 +581,13 @@
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>41</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>42</v>
       </c>
       <c r="D7" s="0" t="s">
         <v>15</v>
@@ -598,13 +595,13 @@
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>44</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>16</v>
@@ -612,44 +609,44 @@
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="12" t="s">
+      <c r="D9" s="0" t="s">
         <v>46</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="12" t="s">
+      <c r="D10" s="0" t="s">
         <v>49</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="12" t="s">
+      <c r="D11" s="0" t="s">
         <v>52</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="12">
@@ -657,13 +654,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="D12" s="0" t="s">
         <v>55</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -671,13 +668,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C13" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="0" t="s">
         <v>57</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="14">
@@ -685,10 +682,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D14" s="0" t="s">
         <v>17</v>
@@ -699,10 +696,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D15" s="0" t="s">
         <v>18</v>
@@ -711,7 +708,7 @@
     <row r="16"/>
     <row r="17">
       <c r="A17" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>

</xml_diff>